<commit_message>
release: version produccion - bot 95% funcional, pendiente extorno y ventas
</commit_message>
<xml_diff>
--- a/ReportesExcel/horario/2026/Julio/MOV_17-07-26.xlsx
+++ b/ReportesExcel/horario/2026/Julio/MOV_17-07-26.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="530" uniqueCount="227">
   <si>
     <t>Nº de Procesado</t>
   </si>
@@ -410,6 +410,291 @@
   </si>
   <si>
     <t>DISTRIBUCION</t>
+  </si>
+  <si>
+    <t>19</t>
+  </si>
+  <si>
+    <t>KS|1|101|6|01|06|1|2|0</t>
+  </si>
+  <si>
+    <t>260053984</t>
+  </si>
+  <si>
+    <t>13:29:39</t>
+  </si>
+  <si>
+    <t>SALIDA</t>
+  </si>
+  <si>
+    <t>06732F05</t>
+  </si>
+  <si>
+    <t>06732F0101</t>
+  </si>
+  <si>
+    <t>20</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|18|2|0</t>
+  </si>
+  <si>
+    <t>001-0040776</t>
+  </si>
+  <si>
+    <t>13:33:06</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|19|2|0</t>
+  </si>
+  <si>
+    <t>001-0040777</t>
+  </si>
+  <si>
+    <t>13:45:43</t>
+  </si>
+  <si>
+    <t>81085172</t>
+  </si>
+  <si>
+    <t>00005878</t>
+  </si>
+  <si>
+    <t>G442</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|20|2|0</t>
+  </si>
+  <si>
+    <t>001-0040778</t>
+  </si>
+  <si>
+    <t>13:47:17</t>
+  </si>
+  <si>
+    <t>81309931</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|21|2|0</t>
+  </si>
+  <si>
+    <t>001-0040779</t>
+  </si>
+  <si>
+    <t>13:48:42</t>
+  </si>
+  <si>
+    <t>01033259</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|22|2|0</t>
+  </si>
+  <si>
+    <t>001-0040780</t>
+  </si>
+  <si>
+    <t>13:49:36</t>
+  </si>
+  <si>
+    <t>25</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|23|2|0</t>
+  </si>
+  <si>
+    <t>001-0040781</t>
+  </si>
+  <si>
+    <t>13:51:37</t>
+  </si>
+  <si>
+    <t>90125019</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|24|2|0</t>
+  </si>
+  <si>
+    <t>175-0007034</t>
+  </si>
+  <si>
+    <t>13:53:36</t>
+  </si>
+  <si>
+    <t>90268207</t>
+  </si>
+  <si>
+    <t>27</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|25|2|0</t>
+  </si>
+  <si>
+    <t>175-0007035</t>
+  </si>
+  <si>
+    <t>13:54:31</t>
+  </si>
+  <si>
+    <t>90495212</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|26|2|0</t>
+  </si>
+  <si>
+    <t>175-0007036</t>
+  </si>
+  <si>
+    <t>13:56:30</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|27|2|0</t>
+  </si>
+  <si>
+    <t>001-0040782</t>
+  </si>
+  <si>
+    <t>13:57:44</t>
+  </si>
+  <si>
+    <t>01036752</t>
+  </si>
+  <si>
+    <t>30</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|28|2|0</t>
+  </si>
+  <si>
+    <t>001-0040783</t>
+  </si>
+  <si>
+    <t>13:59:39</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|29|2|0</t>
+  </si>
+  <si>
+    <t>001-0040784</t>
+  </si>
+  <si>
+    <t>14:00:33</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|30|2|0</t>
+  </si>
+  <si>
+    <t>001-0040785</t>
+  </si>
+  <si>
+    <t>14:01:28</t>
+  </si>
+  <si>
+    <t>33</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|31|2|0</t>
+  </si>
+  <si>
+    <t>001-0040786</t>
+  </si>
+  <si>
+    <t>14:03:36</t>
+  </si>
+  <si>
+    <t>27075119</t>
+  </si>
+  <si>
+    <t>34</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|32|2|0</t>
+  </si>
+  <si>
+    <t>001-0040787</t>
+  </si>
+  <si>
+    <t>14:04:41</t>
+  </si>
+  <si>
+    <t>44958419</t>
+  </si>
+  <si>
+    <t>35</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|33|2|0</t>
+  </si>
+  <si>
+    <t>001-0040788</t>
+  </si>
+  <si>
+    <t>14:05:37</t>
+  </si>
+  <si>
+    <t>00000008</t>
+  </si>
+  <si>
+    <t>36</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|34|2|0</t>
+  </si>
+  <si>
+    <t>001-0040789</t>
+  </si>
+  <si>
+    <t>14:06:34</t>
+  </si>
+  <si>
+    <t>94716306</t>
+  </si>
+  <si>
+    <t>00000009</t>
+  </si>
+  <si>
+    <t>37</t>
+  </si>
+  <si>
+    <t>KS|1|101|1|02|03|35|2|0</t>
+  </si>
+  <si>
+    <t>001-0040790</t>
+  </si>
+  <si>
+    <t>14:07:41</t>
+  </si>
+  <si>
+    <t>33733877</t>
+  </si>
+  <si>
+    <t>00000010</t>
   </si>
 </sst>
 </file>
@@ -462,8 +747,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:W19" totalsRowShown="0">
-  <autoFilter ref="A1:W19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Frame0" displayName="Frame0" ref="A1:W38" totalsRowShown="0">
+  <autoFilter ref="A1:W38"/>
   <tableColumns count="23">
     <tableColumn id="1" name="Nº de Procesado" dataDxfId="0"/>
     <tableColumn id="2" name="Nº correlativo Ksalud" dataDxfId="0"/>
@@ -778,7 +1063,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W19"/>
+  <dimension ref="A1:W38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
@@ -1798,6 +2083,999 @@
         <v>23</v>
       </c>
     </row>
+    <row r="20" spans="1:23">
+      <c r="A20" s="1" t="s">
+        <v>132</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="G20" s="1" t="s">
+        <v>136</v>
+      </c>
+      <c r="H20" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="K20" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="L20" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="M20" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="N20" s="1"/>
+      <c r="O20" s="1"/>
+      <c r="P20" s="1"/>
+      <c r="Q20" s="1"/>
+      <c r="R20" s="1"/>
+      <c r="S20" s="1"/>
+      <c r="T20" s="1"/>
+      <c r="U20" s="1"/>
+      <c r="V20" s="1"/>
+      <c r="W20" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="21" spans="1:23">
+      <c r="A21" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G21" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H21" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+      <c r="K21" s="1"/>
+      <c r="L21" s="1"/>
+      <c r="M21" s="1"/>
+      <c r="N21" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O21" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="P21" s="1"/>
+      <c r="Q21" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="R21" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S21" s="1"/>
+      <c r="T21" s="1"/>
+      <c r="U21" s="1"/>
+      <c r="V21" s="1"/>
+      <c r="W21" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="22" spans="1:23">
+      <c r="A22" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G22" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+      <c r="K22" s="1"/>
+      <c r="L22" s="1"/>
+      <c r="M22" s="1"/>
+      <c r="N22" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O22" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="P22" s="1"/>
+      <c r="Q22" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R22" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S22" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="T22" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="U22" s="1"/>
+      <c r="V22" s="1"/>
+      <c r="W22" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="23" spans="1:23">
+      <c r="A23" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G23" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+      <c r="K23" s="1"/>
+      <c r="L23" s="1"/>
+      <c r="M23" s="1"/>
+      <c r="N23" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O23" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P23" s="1"/>
+      <c r="Q23" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R23" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S23" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="T23" s="1"/>
+      <c r="U23" s="1"/>
+      <c r="V23" s="1"/>
+      <c r="W23" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" spans="1:23">
+      <c r="A24" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>156</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H24" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+      <c r="K24" s="1"/>
+      <c r="L24" s="1"/>
+      <c r="M24" s="1"/>
+      <c r="N24" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O24" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="P24" s="1"/>
+      <c r="Q24" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R24" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="T24" s="1"/>
+      <c r="U24" s="1"/>
+      <c r="V24" s="1"/>
+      <c r="W24" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:23">
+      <c r="A25" s="1" t="s">
+        <v>160</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H25" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="1"/>
+      <c r="M25" s="1"/>
+      <c r="N25" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O25" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="P25" s="1"/>
+      <c r="Q25" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="R25" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S25" s="1"/>
+      <c r="T25" s="1"/>
+      <c r="U25" s="1"/>
+      <c r="V25" s="1"/>
+      <c r="W25" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="26" spans="1:23">
+      <c r="A26" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+      <c r="K26" s="1"/>
+      <c r="L26" s="1"/>
+      <c r="M26" s="1"/>
+      <c r="N26" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O26" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="P26" s="1"/>
+      <c r="Q26" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R26" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S26" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="T26" s="1"/>
+      <c r="U26" s="1"/>
+      <c r="V26" s="1"/>
+      <c r="W26" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:23">
+      <c r="A27" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G27" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+      <c r="K27" s="1"/>
+      <c r="L27" s="1"/>
+      <c r="M27" s="1"/>
+      <c r="N27" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O27" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="P27" s="1"/>
+      <c r="Q27" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R27" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S27" s="1"/>
+      <c r="T27" s="1"/>
+      <c r="U27" s="1"/>
+      <c r="V27" s="1"/>
+      <c r="W27" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="28" spans="1:23">
+      <c r="A28" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>176</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+      <c r="K28" s="1"/>
+      <c r="L28" s="1"/>
+      <c r="M28" s="1"/>
+      <c r="N28" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O28" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="P28" s="1"/>
+      <c r="Q28" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R28" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S28" s="1"/>
+      <c r="T28" s="1"/>
+      <c r="U28" s="1"/>
+      <c r="V28" s="1"/>
+      <c r="W28" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="29" spans="1:23">
+      <c r="A29" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H29" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+      <c r="K29" s="1"/>
+      <c r="L29" s="1"/>
+      <c r="M29" s="1"/>
+      <c r="N29" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O29" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="P29" s="1"/>
+      <c r="Q29" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="R29" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S29" s="1"/>
+      <c r="T29" s="1"/>
+      <c r="U29" s="1"/>
+      <c r="V29" s="1"/>
+      <c r="W29" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="30" spans="1:23">
+      <c r="A30" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>184</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H30" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O30" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R30" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S30" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="T30" s="1"/>
+      <c r="U30" s="1"/>
+      <c r="V30" s="1"/>
+      <c r="W30" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23">
+      <c r="A31" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I31" s="1"/>
+      <c r="J31" s="1"/>
+      <c r="K31" s="1"/>
+      <c r="L31" s="1"/>
+      <c r="M31" s="1"/>
+      <c r="N31" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O31" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="P31" s="1"/>
+      <c r="Q31" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="R31" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S31" s="1"/>
+      <c r="T31" s="1"/>
+      <c r="U31" s="1"/>
+      <c r="V31" s="1"/>
+      <c r="W31" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="32" spans="1:23">
+      <c r="A32" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H32" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O32" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="P32" s="1"/>
+      <c r="Q32" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="R32" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S32" s="1"/>
+      <c r="T32" s="1"/>
+      <c r="U32" s="1"/>
+      <c r="V32" s="1"/>
+      <c r="W32" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="33" spans="1:23">
+      <c r="A33" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O33" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="P33" s="1"/>
+      <c r="Q33" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R33" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S33" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="T33" s="1"/>
+      <c r="U33" s="1"/>
+      <c r="V33" s="1"/>
+      <c r="W33" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:23">
+      <c r="A34" s="1" t="s">
+        <v>200</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H34" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I34" s="1"/>
+      <c r="J34" s="1"/>
+      <c r="K34" s="1"/>
+      <c r="L34" s="1"/>
+      <c r="M34" s="1"/>
+      <c r="N34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O34" s="1" t="s">
+        <v>204</v>
+      </c>
+      <c r="P34" s="1"/>
+      <c r="Q34" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R34" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S34" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="T34" s="1"/>
+      <c r="U34" s="1"/>
+      <c r="V34" s="1"/>
+      <c r="W34" s="1" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="35" spans="1:23">
+      <c r="A35" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>208</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H35" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I35" s="1"/>
+      <c r="J35" s="1"/>
+      <c r="K35" s="1"/>
+      <c r="L35" s="1"/>
+      <c r="M35" s="1"/>
+      <c r="N35" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O35" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="P35" s="1"/>
+      <c r="Q35" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R35" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S35" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="T35" s="1"/>
+      <c r="U35" s="1"/>
+      <c r="V35" s="1"/>
+      <c r="W35" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="36" spans="1:23">
+      <c r="A36" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>212</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H36" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I36" s="1"/>
+      <c r="J36" s="1"/>
+      <c r="K36" s="1"/>
+      <c r="L36" s="1"/>
+      <c r="M36" s="1"/>
+      <c r="N36" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="P36" s="1"/>
+      <c r="Q36" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R36" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S36" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="T36" s="1"/>
+      <c r="U36" s="1"/>
+      <c r="V36" s="1"/>
+      <c r="W36" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="37" spans="1:23">
+      <c r="A37" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H37" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I37" s="1"/>
+      <c r="J37" s="1"/>
+      <c r="K37" s="1"/>
+      <c r="L37" s="1"/>
+      <c r="M37" s="1"/>
+      <c r="N37" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O37" s="1" t="s">
+        <v>219</v>
+      </c>
+      <c r="P37" s="1"/>
+      <c r="Q37" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R37" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S37" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="T37" s="1"/>
+      <c r="U37" s="1"/>
+      <c r="V37" s="1"/>
+      <c r="W37" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="38" spans="1:23">
+      <c r="A38" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>224</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="I38" s="1"/>
+      <c r="J38" s="1"/>
+      <c r="K38" s="1"/>
+      <c r="L38" s="1"/>
+      <c r="M38" s="1"/>
+      <c r="N38" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="O38" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="P38" s="1"/>
+      <c r="Q38" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="R38" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="S38" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="T38" s="1"/>
+      <c r="U38" s="1"/>
+      <c r="V38" s="1"/>
+      <c r="W38" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>